<commit_message>
Added social media extraction
</commit_message>
<xml_diff>
--- a/output/leads.xlsx
+++ b/output/leads.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,26 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>LinkedIn</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Twitter</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Contact Pages</t>
         </is>
       </c>
@@ -468,6 +488,22 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
+          <t>https://www.linkedin.com/company/openai</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/openai/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>https://x.com/OpenAI</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>https://openai.com/about/, https://openai.com/contact-sales/, https://help.openai.com/</t>
         </is>
       </c>
@@ -496,6 +532,18 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
+          <t>https://www.linkedin.com/company/python-software-foundation/</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://twitter.com/ThePSF</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>https://python.org/about/, https://python.org/about/apps/, https://python.org/about/quotes/, https://python.org/about/gettingstarted/, https://python.org/about/help/, https://pyfound.blogspot.com/2026/07/thinking-about-running-for-psf-board.html, https://python.org/about/apps, https://python.org/about/legal/</t>
         </is>
       </c>
@@ -522,7 +570,11 @@
           <t>+1 226-705-2945, +1 650-319-8930, +1 849-936-8072, +33 1 73 01 52 44, +351 21 123 0932, +44 20 3514 6970, +49 89 25552276, +503 2104 5029, +506 4600 8807, +507 839-2268, +51 1 7019264, +55 11 91086-1380, +58 212-7710594, +591 5 0701179, +593 96 428 4222, +595 21 728 9515, +61 1300 748 959, +65 3158 3954</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>https://www.cloudflare.com/resource/contact-enterprise-sales/, https://www.cloudflare.com/about/, https://support.cloudflare.com/</t>
         </is>

</xml_diff>

<commit_message>
Improved company name extraction
</commit_message>
<xml_diff>
--- a/output/leads.xlsx
+++ b/output/leads.xlsx
@@ -495,7 +495,11 @@
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>+1 283-632-2609, +1 306-874-9875, +1 315-780-4138, +1 323-234-3023, +1 331-849-4172, +1 350-362-5418, +1 434-910-6655, +1 530-913-4475, +1 544-251-2325</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>000 example model responses that reflect how patients and clinicians use ChatGPT in the real world. Every few minutes, a physician reviews a new response. Their feedback becomes rubrics and evaluation criteria that help researchers measure whether responses are accurate, safe, clear, complete, appropriately cautious, and useful, 1 critical, 6 high, 1 medium, and 0 low. The main table lists active security findings with titles, categories, severity, and , 30 open-source projects have committed to participate, with initial participants including cURL, Go, Python, Sigstore, and pyca, 5 Instant reaches health performance similar to our latest frontier models on an aggregate of health evaluations, including HealthBench Professional, substantia, 5 Instant responses as having fewer failure modes than those from older models and physicians. For example, GPT-5.5 Instant had fewer instances of not tailoring to local healthcare context, missing red flags or referral to care, or failing, 5 nerve root, for example, the MRI ca, 6 Sol is better at helping people find and fix vulnerabilities than reliably carrying out end-to-end attacks. As these capabilities continue to advance, our priority is to make sure they reach and benefit defenders, who can use these tools to find weaknesses, develop patches, and streng, 6 Sol is our strongest model yet. To give a preview of model performance, we share a set of evaluations highlighting improved agentic capabilities in coding, biology, and cybersecurity, with addit, 6 Sol launches with our most robust safety stack to date. We strengthened protections for higher-risk activity, sensitive cyber requests, and repeated misuse, and spent multiple weeks finding weaknesses, pressure, 6 Sol, Terra and Luna with our most robust safeguards to date, with confi, 6 Sol, Terra, and Luna g, 6 Sol, Terra, and Luna m, 6 Sol, a next-generation model with stronger capabilities in coding, science, and cybersecurity, paired wit, 6 models will initially be available through the API and Codex to a select group of trusted partners and organizations. We plan to make them more broadly available to people using ChatGPT, Codex, and the AP, 6 preview, we use layered safeguards, with exact configurations varying across models, and pressure-test them for real-world attacks. These include protections trained into the model, real-time checks during generation, account-level signals, differentiated access, monitoring, enforcement, and contin</t>
@@ -557,19 +561,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.cloudflare.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Cloudflare: Build for the agent era</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.cloudflare.com</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Cloudflare: Build for the agent era</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>dpo@cloudflare.com, privacyquestions@cloudflare.com, sar@cloudflare.com, unsubscribe@cloudflare.com</t>
@@ -577,7 +581,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+1 226-705-2945, +1 650-319-8930, +1 849-936-8072, +33 1 73 01 52 44, +351 21 123 0932, +44 20 3514 6970, +49 89 25552276, +503 2104 5029, +506 4600 8807, +507 839-2268, +51 1 7019264, +55 11 91086-1380, +58 212-7710594, +591 5 0701179, +593 96 428 4222, +595 21 728 9515, +61 1300 748 959, +65 3158 3954</t>
+          <t>+1 226-705-2945, +1 354-811-7155, +1 650-319-8930, +1 800-301-4062, +1 849-936-8072, +12267052945, +16503198930, +18499368072, +188899, +33 1 73 01 52 44, +33173015244, +351 21 123 0932, +351211230932, +44 20 3514 6970, +442035146970, +49 89 25552276, +498925552276, +503 2104 5029, +50321045029, +50422630049, +506 4600 8807, +50646008807, +507 839-2268, +5078392268, +51 1 7019264, +5117019264, +55 11 91086-1380, +5511910861380, +58 212-7710594, +582127710594, +591 5 0701179, +59150701179, +593 96 428 4222, +593964284222, +595 21 728 9515, +595217289515, +61 1300 748 959, +611300748959, +65 3158 3954, +6531583954, 0008000501996, 00180349248340049, 00798142030192, 0080049240880219, 00801491427, 018005190085, 020260652, 0208090009, 05017911110, 08002220652, 180013120014, 1800819200, 30083639, 4000280226, 4054318, 69906420, 8000120099, 8000770774, 800088840, 8003014062, 800630141, 800914282, 800959181, 900943467</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">

</xml_diff>

<commit_message>
Scanning files and website scrapping
</commit_message>
<xml_diff>
--- a/output/leads.xlsx
+++ b/output/leads.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -481,71 +481,72 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>403 Forbidden</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://openai.com</t>
+          <t>https://publicserviceplumbers.com/?utm_source=google-gbp&amp;utm_medium=organic&amp;utm_campaign=*163*public-service-plumbers-dallas</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>OpenAI | Research &amp; Deployment</t>
+          <t>403 Forbidden</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>+1 283-632-2609, +1 306-874-9875, +1 315-780-4138, +1 323-234-3023, +1 331-849-4172, +1 350-362-5418, +1 434-910-6655, +1 530-913-4475, +1 544-251-2325</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>000 example model responses that reflect how patients and clinicians use ChatGPT in the real world. Every few minutes, a physician reviews a new response. Their feedback becomes rubrics and evaluation criteria that help researchers measure whether responses are accurate, safe, clear, complete, appropriately cautious, and useful, 1 critical, 6 high, 1 medium, and 0 low. The main table lists active security findings with titles, categories, severity, and , 30 open-source projects have committed to participate, with initial participants including cURL, Go, Python, Sigstore, and pyca, 5 Instant reaches health performance similar to our latest frontier models on an aggregate of health evaluations, including HealthBench Professional, substantia, 5 Instant responses as having fewer failure modes than those from older models and physicians. For example, GPT-5.5 Instant had fewer instances of not tailoring to local healthcare context, missing red flags or referral to care, or failing, 5 nerve root, for example, the MRI ca, 6 Sol is better at helping people find and fix vulnerabilities than reliably carrying out end-to-end attacks. As these capabilities continue to advance, our priority is to make sure they reach and benefit defenders, who can use these tools to find weaknesses, develop patches, and streng, 6 Sol is our strongest model yet. To give a preview of model performance, we share a set of evaluations highlighting improved agentic capabilities in coding, biology, and cybersecurity, with addit, 6 Sol launches with our most robust safety stack to date. We strengthened protections for higher-risk activity, sensitive cyber requests, and repeated misuse, and spent multiple weeks finding weaknesses, pressure, 6 Sol, Terra and Luna with our most robust safeguards to date, with confi, 6 Sol, Terra, and Luna g, 6 Sol, Terra, and Luna m, 6 Sol, a next-generation model with stronger capabilities in coding, science, and cybersecurity, paired wit, 6 models will initially be available through the API and Codex to a select group of trusted partners and organizations. We plan to make them more broadly available to people using ChatGPT, Codex, and the AP, 6 preview, we use layered safeguards, with exact configurations varying across models, and pressure-test them for real-world attacks. These include protections trained into the model, real-time checks during generation, account-level signals, differentiated access, monitoring, enforcement, and contin</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Cloudflare, Next.js</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>https://openai.com/about/, https://openai.com/news/company-announcements/, https://openai.com/security-and-privacy/, https://openai.com/contact-sales/, https://openai.com/careers/</t>
-        </is>
-      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Python.org</t>
+          <t>Metro Flow Plumbing - Dallas Emergency Plumbers</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://python.org</t>
+          <t>https://metroflowplumbing.com/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Welcome to Python.org</t>
+          <t>Expert Plumbing Services | Dallas, TX | Metro Flow Plumbing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>psf@python.org, python-announce@python.org, webmaster@python.org</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+          <t>info@construction.com, metroflow@metroflowplumbing.com</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>+1 214-214-4718, +1 214-328-7371, +1 681-613-3838, +1 928-619-2192, 214-328-7371</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>30 years.
+Our team consists of licensed, certified, and insure, 323 Point Inspection
+The Highest Level of Dallas Plumbing Valet Service
+Our exclusive offerings have resulted in tremendous customer satisfaction. As one satisfied customer, Emma Vernon, stated, 50 discount on services or the benefits from our Diamond Club membership, must be used independently to maintain the integrity of each promotion.
+Many of our customers appreciate the value of our services, as highlighted by Dorothy Woodward, who lauded, 7 emergency assistance to ensure that your plumbing issues are addressed promptly and efficiently, no matter the time of day or night. Our team of certified, insured, and highly trained plumbers are ready to tackle any emergency situation, from burst, 7 to address your urgent plumbing needs, ensuring you receive prompt and effective service. In fact, we often have a crew onsite within an hour of your call.
+We prioritize your emergencies, offering a warm voice, a courteous call, and a seam</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Cloudflare, Squarespace, WordPress</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -554,53 +555,133 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://python.org/about/, https://python.org/about/apps/, https://python.org/about/quotes/, https://python.org/about/gettingstarted/, https://python.org/about/help/</t>
+          <t>https://metroflowplumbing.com/about/, https://metroflowplumbing.com/career, https://metroflowplumbing.com/contact/, https://metroflowplumbing.com/#contact, https://metroflowplumbing.com/privacy-policy/</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Cloudflare</t>
+          <t>Dallas Plumbing &amp; Air Conditioning</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.cloudflare.com</t>
+          <t>https://www.dallasplumbing.com/dallas/?utm_source=organic&amp;utm_medium=organic&amp;utm_campaign=dallas&amp;utm_id=gbp</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cloudflare: Build for the agent era</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>dpo@cloudflare.com, privacyquestions@cloudflare.com, sar@cloudflare.com, unsubscribe@cloudflare.com</t>
-        </is>
-      </c>
+          <t>Plumber &amp; HVAC Company | Dallas, TX | Dallas Plumbing &amp; AC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+1 226-705-2945, +1 354-811-7155, +1 650-319-8930, +1 800-301-4062, +1 849-936-8072, +12267052945, +16503198930, +18499368072, +188899, +33 1 73 01 52 44, +33173015244, +351 21 123 0932, +351211230932, +44 20 3514 6970, +442035146970, +49 89 25552276, +498925552276, +503 2104 5029, +50321045029, +50422630049, +506 4600 8807, +50646008807, +507 839-2268, +5078392268, +51 1 7019264, +5117019264, +55 11 91086-1380, +5511910861380, +58 212-7710594, +582127710594, +591 5 0701179, +59150701179, +593 96 428 4222, +593964284222, +595 21 728 9515, +595217289515, +61 1300 748 959, +611300748959, +65 3158 3954, +6531583954, 0008000501996, 00180349248340049, 00798142030192, 0080049240880219, 00801491427, 018005190085, 020260652, 0208090009, 05017911110, 08002220652, 180013120014, 1800819200, 30083639, 4000280226, 4054318, 69906420, 8000120099, 8000770774, 800088840, 8003014062, 800630141, 800914282, 800959181, 900943467</t>
+          <t>${phoneNumber.replace(/[()\s-]/g,, +1 214-227-9459, +1 239-207-8228, +1 469-936-0899, 2142279459, 4699360899</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 Application, which is not covered by this Policy, are somewh, 1 Kyobashi, Chuo-ku, Tokyo, 104, 1 World Trade Center, 88th Floor, New York, NY 10007, 1 World Trade Center, 88th Floor, New York, NY 10007 , 1 resolver with any other Cloudflare or third party data in any way that can be used to identify individual end users. Cloudflare may store aggregated data, as outlined within our 1.1.1.1 resolver commitments to privacy, indefinitely in order to power Cloudflare Radar and assist Cloudflare in improving Cloudflare services, such as, enhancing , 101 Townsend St., San Francisco, CA 94107, 15 minutes to get up and running. The ability to quickly spin up a Worker, deploy it to production, and scale , 16 South Guangshun Street, Donghuang Building 17th Floor, Chaoyang District, Beijing 10, 2 has been the glue behind our multi-cloud architecture for training and processing requests. We are now able to store our training and production data in R2 for access by any cloud, without egress fees, and get th, 301 N Neil St Suite 440, Champaign, IL 61820, 301 N Neil St Suite 440, Champaign, IL 61820 , 388 George Street, Sydney, NSW 2000 , 900 19th Street, N.W., Suite 375, Washington, DC 20006, 900 19th Street, N.W., Suite 375, Washington, DC 20006 </t>
+          <t>120 years after its founding, Dallas Plumbing Company continues to serve homes and businesses across North Texas, combining old-fashioned customer service with modern expertise in plumbing, heating, and air co</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Astro, Cloudflare</t>
+          <t>WordPress</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>https://www.cloudflare.com/resource/contact-enterprise-sales/, https://www.cloudflare.com/about/, https://www.cloudflare.com/careers/, https://www.cloudflare.com/policies/privacy/</t>
+      <c r="L4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Dallas Plumber</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://callmilestone.com/dallas/plumbing/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Dallas Plumber - Voted The Best Plumbing Service in Dallas, TX!</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>contact-us@callmilestone.com, media@callmilestone.com, optout@callmilestone.com, recruiting@callmilestone.com</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>%202142672405, %202147176708, +1 208-558-2039, +1 214-216-0387, +1 214-267-2405, +1 214-348-5100, +1 214-717-6708, +1 501-960-7843, +1 707-893-3078, +1 817-267-2405, +1 817-672-8166, +1 972-913-6165, +247 42475, 214-348-5100, 2142672405, 2143485100, 2147176708, 8172672405</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1920 Hutton Ct Suite 200, Farmers Branch, TX 75234, 2360 Crist Rd Suite B900, Garland, TX 75040, 2801 N Central Expy, Plano, TX 75075, 401 West Interstate 30, Garland, TX 75043, 4651 W John Carpenter Fwy Suite 170, Irving, TX 75063, 5414 Forest Ln, Dallas, TX 75229, 5414 Forest Ln, Dallas, TX 75229 , 5535 Airport Fwy Unit A, Haltom City, TX 76117, 600 W 6th St Ste 470, Fort Worth, TX 76102, 701 E Walnut St, Garland, TX 75040, 701 E Walnut St, Garland, TX 75040 </t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>WordPress</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://callmilestone.com/about-us/, https://callmilestone.com/careers/, https://callmilestone.com/privacy-policy/, https://callmilestone.com/contact-us/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tribeca Plumbing, Inc.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.tribecaplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Plumbing, Electrical, and HVAC Services in Dallas, TX | Tribeca Plumbing, Inc.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>(214) 402-5454, +1 214-402-5454, +1 327-825-8120, +1 329-232-6620, +1 329-253-2400, +1 329-332-9460, +1 329-666-7480, +1 971-958-1450, 2144025454</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>5454 For Fast and Reliable Plumbing Services in Dallas, TX and the Surrounding Areas From Tribeca Plumbing, Inc</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Cloudflare, WordPress</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://www.tribecaplumbinginc.com/about-us/, https://www.tribecaplumbinginc.com/careers/, https://www.tribecaplumbinginc.com/hvac-services/heating-services-company/, https://www.tribecaplumbinginc.com/contact-us/, https://www.tribecaplumbinginc.com/privacy-policy/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactored scanner into service architecture
</commit_message>
<xml_diff>
--- a/output/leads.xlsx
+++ b/output/leads.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -559,132 +559,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Dallas Plumbing &amp; Air Conditioning</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://www.dallasplumbing.com/dallas/?utm_source=organic&amp;utm_medium=organic&amp;utm_campaign=dallas&amp;utm_id=gbp</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Plumber &amp; HVAC Company | Dallas, TX | Dallas Plumbing &amp; AC</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>${phoneNumber.replace(/[()\s-]/g,, +1 214-227-9459, +1 239-207-8228, +1 469-936-0899, 2142279459, 4699360899</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>120 years after its founding, Dallas Plumbing Company continues to serve homes and businesses across North Texas, combining old-fashioned customer service with modern expertise in plumbing, heating, and air co</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>WordPress</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
-      <c r="L4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Dallas Plumber</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>https://callmilestone.com/dallas/plumbing/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Dallas Plumber - Voted The Best Plumbing Service in Dallas, TX!</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>contact-us@callmilestone.com, media@callmilestone.com, optout@callmilestone.com, recruiting@callmilestone.com</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>%202142672405, %202147176708, +1 208-558-2039, +1 214-216-0387, +1 214-267-2405, +1 214-348-5100, +1 214-717-6708, +1 501-960-7843, +1 707-893-3078, +1 817-267-2405, +1 817-672-8166, +1 972-913-6165, +247 42475, 214-348-5100, 2142672405, 2143485100, 2147176708, 8172672405</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1920 Hutton Ct Suite 200, Farmers Branch, TX 75234, 2360 Crist Rd Suite B900, Garland, TX 75040, 2801 N Central Expy, Plano, TX 75075, 401 West Interstate 30, Garland, TX 75043, 4651 W John Carpenter Fwy Suite 170, Irving, TX 75063, 5414 Forest Ln, Dallas, TX 75229, 5414 Forest Ln, Dallas, TX 75229 , 5535 Airport Fwy Unit A, Haltom City, TX 76117, 600 W 6th St Ste 470, Fort Worth, TX 76102, 701 E Walnut St, Garland, TX 75040, 701 E Walnut St, Garland, TX 75040 </t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>WordPress</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>https://callmilestone.com/about-us/, https://callmilestone.com/careers/, https://callmilestone.com/privacy-policy/, https://callmilestone.com/contact-us/</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Tribeca Plumbing, Inc.</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>https://www.tribecaplumbinginc.com/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Plumbing, Electrical, and HVAC Services in Dallas, TX | Tribeca Plumbing, Inc.</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>(214) 402-5454, +1 214-402-5454, +1 327-825-8120, +1 329-232-6620, +1 329-253-2400, +1 329-332-9460, +1 329-666-7480, +1 971-958-1450, 2144025454</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>5454 For Fast and Reliable Plumbing Services in Dallas, TX and the Surrounding Areas From Tribeca Plumbing, Inc</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Cloudflare, WordPress</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>https://www.tribecaplumbinginc.com/about-us/, https://www.tribecaplumbinginc.com/careers/, https://www.tribecaplumbinginc.com/hvac-services/heating-services-company/, https://www.tribecaplumbinginc.com/contact-us/, https://www.tribecaplumbinginc.com/privacy-policy/</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor architecture, optimize crawling, add lead qualification
</commit_message>
<xml_diff>
--- a/output/leads.xlsx
+++ b/output/leads.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LeadGen Pro" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'LeadGen Pro'!$A$1:$L$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +27,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +57,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,66 +427,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Company</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Website</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Emails</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Phones</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Addresses</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Facebook</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Instagram</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Twitter</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Contact Pages</t>
         </is>
@@ -481,72 +509,71 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>403 Forbidden</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://publicserviceplumbers.com/?utm_source=google-gbp&amp;utm_medium=organic&amp;utm_campaign=*163*public-service-plumbers-dallas</t>
+          <t>https://openai.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>403 Forbidden</t>
+          <t>OpenAI | Research &amp; Deployment</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>+1 283-632-2609, +1 306-874-9875, +1 315-780-4138, +1 323-234-3023, +1 331-849-4172, +1 350-362-5418, +1 434-910-6655, +1 530-913-4475, +1 544-251-2325</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>000 example model responses that reflect how patients and clinicians use ChatGPT in the real world. Every few minutes, a physician reviews a new response. Their feedback becomes rubrics and evaluation criteria that help researchers measure whether responses are accurate, safe, clear, complete, appropriately cautious, and useful, 1 critical, 6 high, 1 medium, and 0 low. The main table lists active security findings with titles, categories, severity, and , 2 Type 2 examination of controls relevant to Security, Availability, Confidentiality, and Privac, 2019 certifications for the information security and privacy management systems supporting the OpenAI API, ChatGPT Enterprise, and ChatGP, 30 open-source projects have committed to participate, with initial participants including cURL, Go, Python, Sigstore, and pyca, 5 Instant reaches health performance similar to our latest frontier models on an aggregate of health evaluations, including HealthBench Professional, substantia, 5 Instant responses as having fewer failure modes than those from older models and physicians. For example, GPT-5.5 Instant had fewer instances of not tailoring to local healthcare context, missing red flags or referral to care, or failing, 5 nerve root, for example, the MRI ca, 6 Sol is better at helping people find and fix vulnerabilities than reliably carrying out end-to-end attacks. As these capabilities continue to advance, our priority is to make sure they reach and benefit defenders, who can use these tools to find weaknesses, develop patches, and streng, 6 Sol is our strongest model yet. To give a preview of model performance, we share a set of evaluations highlighting improved agentic capabilities in coding, biology, and cybersecurity, with addit, 6 Sol launches with our most robust safety stack to date. We strengthened protections for higher-risk activity, sensitive cyber requests, and repeated misuse, and spent multiple weeks finding weaknesses, pressure, 6 Sol, Terra and Luna with our most robust safeguards to date, with confi, 6 Sol, Terra, and Luna g, 6 Sol, Terra, and Luna m, 6 Sol, a next-generation model with stronger capabilities in coding, science, and cybersecurity, paired wit, 6 models will initially be available through the API and Codex to a select group of trusted partners and organizations. We plan to make them more broadly available to people using ChatGPT, Codex, and the AP, 6 preview, we use layered safeguards, with exact configurations varying across models, and pressure-test them for real-world attacks. These include protections trained into the model, real-time checks during generation, account-level signals, differentiated access, monitoring, enforcement, and contin</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Cloudflare, Next.js</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://openai.com/about/, https://openai.com/news/company-announcements/, https://openai.com/security-and-privacy/, https://openai.com/contact-sales/, https://openai.com/careers/</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Metro Flow Plumbing - Dallas Emergency Plumbers</t>
+          <t>Python.org</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://metroflowplumbing.com/</t>
+          <t>https://python.org</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Expert Plumbing Services | Dallas, TX | Metro Flow Plumbing</t>
+          <t>Welcome to Python.org</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>info@construction.com, metroflow@metroflowplumbing.com</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>+1 214-214-4718, +1 214-328-7371, +1 681-613-3838, +1 928-619-2192, 214-328-7371</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>30 years.
-Our team consists of licensed, certified, and insure, 323 Point Inspection
-The Highest Level of Dallas Plumbing Valet Service
-Our exclusive offerings have resulted in tremendous customer satisfaction. As one satisfied customer, Emma Vernon, stated, 50 discount on services or the benefits from our Diamond Club membership, must be used independently to maintain the integrity of each promotion.
-Many of our customers appreciate the value of our services, as highlighted by Dorothy Woodward, who lauded, 7 emergency assistance to ensure that your plumbing issues are addressed promptly and efficiently, no matter the time of day or night. Our team of certified, insured, and highly trained plumbers are ready to tackle any emergency situation, from burst, 7 to address your urgent plumbing needs, ensuring you receive prompt and effective service. In fact, we often have a crew onsite within an hour of your call.
-We prioritize your emergencies, offering a warm voice, a courteous call, and a seam</t>
-        </is>
-      </c>
+          <t>psf&amp;#64;python.org, python-announce&amp;#64;python.org, webmaster&amp;#64;python.org</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Cloudflare, Squarespace, WordPress</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -555,11 +582,58 @@
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://metroflowplumbing.com/about/, https://metroflowplumbing.com/career, https://metroflowplumbing.com/contact/, https://metroflowplumbing.com/#contact, https://metroflowplumbing.com/privacy-policy/</t>
+          <t>https://python.org/about/, https://python.org/about/apps/, https://python.org/about/quotes/, https://python.org/about/gettingstarted/, https://python.org/about/help/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://cloudflare.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cloudflare: Build for the agent era</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>dpo@cloudflare.com, privacyquestions@cloudflare.com, sar@cloudflare.com, unsubscribe@cloudflare.com</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>+1 226-705-2945, +1 354-811-7155, +1 650-319-8930, +1 800-301-4062, +1 849-936-8072, +12267052945, +16503198930, +18499368072, +188899, +33 1 73 01 52 44, +33173015244, +351 21 123 0932, +351211230932, +44 20 3514 6970, +442035146970, +49 89 25552276, +498925552276, +503 2104 5029, +50321045029, +50422630049, +506 4600 8807, +50646008807, +507 839-2268, +5078392268, +51 1 7019264, +5117019264, +55 11 91086-1380, +5511910861380, +58 212-7710594, +582127710594, +591 5 0701179, +59150701179, +593 96 428 4222, +593964284222, +595 21 728 9515, +595217289515, +61 1300 748 959, +611300748959, +65 3158 3954, +6531583954, 0008000501996, 00180349248340049, 00798142030192, 0080049240880219, 00801491427, 018005190085, 020260652, 0208090009, 05017911110, 08002220652, 180013120014, 1800819200, 30083639, 4000280226, 4054318, 69906420, 8000120099, 8000770774, 800088840, 8003014062, 800630141, 800914282, 800959181, 900943467</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 Application, which is not covered by this Policy, are somewh, 1 Kyobashi, Chuo-ku, Tokyo, 104, 1 World Trade Center, 88th Floor, New York, NY 10007, 1 World Trade Center, 88th Floor, New York, NY 10007 , 1 resolver with any other Cloudflare or third party data in any way that can be used to identify individual end users. Cloudflare may store aggregated data, as outlined within our 1.1.1.1 resolver commitments to privacy, indefinitely in order to power Cloudflare Radar and assist Cloudflare in improving Cloudflare services, such as, enhancing , 101 Townsend St., San Francisco, CA 94107, 15 minutes to get up and running. The ability to quickly spin up a Worker, deploy it to production, and scale , 16 South Guangshun Street, Donghuang Building 17th Floor, Chaoyang District, Beijing 10, 2 has been the glue behind our multi-cloud architecture for training and processing requests. We are now able to store our training and production data in R2 for access by any cloud, without egress fees, and get th, 301 N Neil St Suite 440, Champaign, IL 61820, 301 N Neil St Suite 440, Champaign, IL 61820 , 388 George Street, Sydney, NSW 2000 , 900 19th Street, N.W., Suite 375, Washington, DC 20006, 900 19th Street, N.W., Suite 375, Washington, DC 20006 </t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Astro, Cloudflare</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://cloudflare.com/resource/contact-enterprise-sales/, https://cloudflare.com/about/, https://cloudflare.com/careers/, https://cloudflare.com/policies/privacy/</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Start email ranking engine
</commit_message>
<xml_diff>
--- a/output/leads.xlsx
+++ b/output/leads.xlsx
@@ -528,11 +528,7 @@
           <t>+1 283-632-2609, +1 306-874-9875, +1 315-780-4138, +1 323-234-3023, +1 331-849-4172, +1 350-362-5418, +1 434-910-6655, +1 530-913-4475, +1 544-251-2325</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>000 example model responses that reflect how patients and clinicians use ChatGPT in the real world. Every few minutes, a physician reviews a new response. Their feedback becomes rubrics and evaluation criteria that help researchers measure whether responses are accurate, safe, clear, complete, appropriately cautious, and useful, 1 critical, 6 high, 1 medium, and 0 low. The main table lists active security findings with titles, categories, severity, and , 2 Type 2 examination of controls relevant to Security, Availability, Confidentiality, and Privac, 2019 certifications for the information security and privacy management systems supporting the OpenAI API, ChatGPT Enterprise, and ChatGP, 30 open-source projects have committed to participate, with initial participants including cURL, Go, Python, Sigstore, and pyca, 5 Instant reaches health performance similar to our latest frontier models on an aggregate of health evaluations, including HealthBench Professional, substantia, 5 Instant responses as having fewer failure modes than those from older models and physicians. For example, GPT-5.5 Instant had fewer instances of not tailoring to local healthcare context, missing red flags or referral to care, or failing, 5 nerve root, for example, the MRI ca, 6 Sol is better at helping people find and fix vulnerabilities than reliably carrying out end-to-end attacks. As these capabilities continue to advance, our priority is to make sure they reach and benefit defenders, who can use these tools to find weaknesses, develop patches, and streng, 6 Sol is our strongest model yet. To give a preview of model performance, we share a set of evaluations highlighting improved agentic capabilities in coding, biology, and cybersecurity, with addit, 6 Sol launches with our most robust safety stack to date. We strengthened protections for higher-risk activity, sensitive cyber requests, and repeated misuse, and spent multiple weeks finding weaknesses, pressure, 6 Sol, Terra and Luna with our most robust safeguards to date, with confi, 6 Sol, Terra, and Luna g, 6 Sol, Terra, and Luna m, 6 Sol, a next-generation model with stronger capabilities in coding, science, and cybersecurity, paired wit, 6 models will initially be available through the API and Codex to a select group of trusted partners and organizations. We plan to make them more broadly available to people using ChatGPT, Codex, and the AP, 6 preview, we use layered safeguards, with exact configurations varying across models, and pressure-test them for real-world attacks. These include protections trained into the model, real-time checks during generation, account-level signals, differentiated access, monitoring, enforcement, and contin</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Cloudflare, Next.js</t>
@@ -566,7 +562,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>psf&amp;#64;python.org, python-announce&amp;#64;python.org, webmaster&amp;#64;python.org</t>
+          <t>psf@python.org, python-announce@python.org, webmaster@python.org</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -604,17 +600,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>dpo@cloudflare.com, privacyquestions@cloudflare.com, sar@cloudflare.com, unsubscribe@cloudflare.com</t>
+          <t>dpo@cloudflare.com, homepage@cloudflare.com, privacyquestions@cloudflare.com, record@cloudflare.com, sar@cloudflare.com, unsubscribe@cloudflare.com</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>+1 226-705-2945, +1 650-319-8930, +1 800-301-4062, +1 849-936-8072, +12267052945, +16503198930, +18499368072, +188899, +33 1 73 01 52 44, +33173015244, +351 21 123 0932, +351211230932, +44 20 3514 6970, +442035146970, +49 89 25552276, +498925552276, +503 2104 5029, +50321045029, +50422630049, +506 4600 8807, +50646008807, +507 839-2268, +5078392268, +51 1 7019264, +5117019264, +55 11 91086-1380, +5511910861380, +58 212-7710594, +582127710594, +591 5 0701179, +59150701179, +593 96 428 4222, +593964284222, +595 21 728 9515, +595217289515, +61 1300 748 959, +611300748959, +65 3158 3954, +6531583954, 0008000501996, 00180349248340049, 00798142030192, 0080049240880219, 00801491427, 018005190085, 020260652, 0208090009, 05017911110, 08002220652, 180013120014, 1800819200, 30083639, 4000280226, 4054318, 69906420, 8000120099, 8000770774, 800088840, 8003014062, 800630141, 800914282, 800959181, 900943467</t>
+          <t>+1 226-705-2945, +1 354-811-7155, +1 650-319-8930, +1 800-301-4062, +1 849-936-8072, +33 1 73 01 52 44, +351 21 123 0932, +44 20 3514 6970, +49 89 25552276, +503 2104 5029, +506 4600 8807, +507 839-2268, +51 1 7019264, +55 11 91086-1380, +58 212-7710594, +591 5 0701179, +593 96 428 4222, +595 21 728 9515, +61 1300 748 959, +65 3158 3954</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 Application, which is not covered by this Policy, are somewh, 1 Kyobashi, Chuo-ku, Tokyo, 104, 1 World Trade Center, 88th Floor, New York, NY 10007, 1 World Trade Center, 88th Floor, New York, NY 10007 , 1 resolver with any other Cloudflare or third party data in any way that can be used to identify individual end users. Cloudflare may store aggregated data, as outlined within our 1.1.1.1 resolver commitments to privacy, indefinitely in order to power Cloudflare Radar and assist Cloudflare in improving Cloudflare services, such as, enhancing , 101 Townsend St., San Francisco, CA 94107, 15 minutes to get up and running. The ability to quickly spin up a Worker, deploy it to production, and scale , 16 South Guangshun Street, Donghuang Building 17th Floor, Chaoyang District, Beijing 10, 2 has been the glue behind our multi-cloud architecture for training and processing requests. We are now able to store our training and production data in R2 for access by any cloud, without egress fees, and get th, 301 N Neil St Suite 440, Champaign, IL 61820, 301 N Neil St Suite 440, Champaign, IL 61820 , 388 George Street, Sydney, NSW 2000 , 900 19th Street, N.W., Suite 375, Washington, DC 20006, 900 19th Street, N.W., Suite 375, Washington, DC 20006 </t>
+          <t>101 Townsend St. San Francisco, CA 94107 Austin 405 Comal St. Austin, TX 78702, 101 Townsend St., San Francisco, CA 94107, 301 N Neil St Suite 440, Champaign, IL 61820</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">

</xml_diff>